<commit_message>
start fixing EE capacity bug
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/data_case_russia_BASE.xlsx
+++ b/01_data/01_input_data/02_processed/data_case_russia_BASE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2D37504-4442-4B67-8535-97C4CF4EEA6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1566B27A-FE11-4B38-9184-229B3678B3DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="4" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1558" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1574" uniqueCount="98">
   <si>
     <t>Commodities</t>
   </si>
@@ -1151,7 +1151,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA366CBE-E84C-4E05-9B58-54F3A95EEAB7}">
-  <dimension ref="A1:B140"/>
+  <dimension ref="A1:B142"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -2148,129 +2148,145 @@
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="B125" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="B126" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B127" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B128" t="s">
-        <v>16</v>
+        <v>82</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B129" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B130" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B131" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B132" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B133" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B134" t="s">
-        <v>66</v>
+        <v>18</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B135" t="s">
-        <v>59</v>
+        <v>20</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B136" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B137" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B138" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B139" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
+        <v>94</v>
+      </c>
+      <c r="B140" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A141" t="s">
+        <v>95</v>
+      </c>
+      <c r="B141" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A142" t="s">
         <v>96</v>
       </c>
-      <c r="B140" t="s">
+      <c r="B142" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2281,7 +2297,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C781A78E-EFEC-4F2E-A496-3B44BD173FD3}">
-  <dimension ref="A1:I281"/>
+  <dimension ref="A1:I285"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -6375,19 +6391,19 @@
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B142" t="s">
-        <v>15</v>
+        <v>97</v>
       </c>
       <c r="C142" t="s">
-        <v>16</v>
+        <v>72</v>
       </c>
       <c r="D142">
-        <v>10000</v>
+        <v>24.424999999999997</v>
       </c>
       <c r="E142">
-        <v>10000</v>
+        <v>24.424999999999997</v>
       </c>
       <c r="F142">
         <v>1</v>
@@ -6396,7 +6412,7 @@
         <v>10000000</v>
       </c>
       <c r="H142">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I142">
         <v>1</v>
@@ -6404,19 +6420,19 @@
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B143" t="s">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="C143" t="s">
-        <v>18</v>
+        <v>97</v>
       </c>
       <c r="D143">
-        <v>10000</v>
+        <v>24.424999999999997</v>
       </c>
       <c r="E143">
-        <v>10000</v>
+        <v>24.424999999999997</v>
       </c>
       <c r="F143">
         <v>1</v>
@@ -6425,7 +6441,7 @@
         <v>10000000</v>
       </c>
       <c r="H143">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I143">
         <v>1</v>
@@ -6436,10 +6452,10 @@
         <v>12</v>
       </c>
       <c r="B144" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C144" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D144">
         <v>10000</v>
@@ -6465,10 +6481,10 @@
         <v>12</v>
       </c>
       <c r="B145" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C145" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D145">
         <v>10000</v>
@@ -6494,10 +6510,10 @@
         <v>12</v>
       </c>
       <c r="B146" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C146" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D146">
         <v>10000</v>
@@ -6523,10 +6539,10 @@
         <v>12</v>
       </c>
       <c r="B147" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C147" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D147">
         <v>10000</v>
@@ -6552,10 +6568,10 @@
         <v>12</v>
       </c>
       <c r="B148" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C148" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D148">
         <v>10000</v>
@@ -6581,10 +6597,10 @@
         <v>12</v>
       </c>
       <c r="B149" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C149" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D149">
         <v>10000</v>
@@ -6610,10 +6626,10 @@
         <v>12</v>
       </c>
       <c r="B150" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C150" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D150">
         <v>10000</v>
@@ -6639,10 +6655,10 @@
         <v>12</v>
       </c>
       <c r="B151" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C151" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D151">
         <v>10000</v>
@@ -6668,10 +6684,10 @@
         <v>12</v>
       </c>
       <c r="B152" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C152" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D152">
         <v>10000</v>
@@ -6697,10 +6713,10 @@
         <v>12</v>
       </c>
       <c r="B153" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C153" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D153">
         <v>10000</v>
@@ -6726,10 +6742,10 @@
         <v>12</v>
       </c>
       <c r="B154" t="s">
-        <v>78</v>
+        <v>35</v>
       </c>
       <c r="C154" t="s">
-        <v>77</v>
+        <v>36</v>
       </c>
       <c r="D154">
         <v>10000</v>
@@ -6755,10 +6771,10 @@
         <v>12</v>
       </c>
       <c r="B155" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C155" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D155">
         <v>10000</v>
@@ -6784,10 +6800,10 @@
         <v>12</v>
       </c>
       <c r="B156" t="s">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="C156" t="s">
-        <v>42</v>
+        <v>77</v>
       </c>
       <c r="D156">
         <v>10000</v>
@@ -6813,10 +6829,10 @@
         <v>12</v>
       </c>
       <c r="B157" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C157" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="D157">
         <v>10000</v>
@@ -6842,10 +6858,10 @@
         <v>12</v>
       </c>
       <c r="B158" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C158" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D158">
         <v>10000</v>
@@ -6871,10 +6887,10 @@
         <v>12</v>
       </c>
       <c r="B159" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C159" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="D159">
         <v>10000</v>
@@ -6900,10 +6916,10 @@
         <v>12</v>
       </c>
       <c r="B160" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C160" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D160">
         <v>10000</v>
@@ -6929,10 +6945,10 @@
         <v>12</v>
       </c>
       <c r="B161" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C161" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D161">
         <v>10000</v>
@@ -6958,10 +6974,10 @@
         <v>12</v>
       </c>
       <c r="B162" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C162" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D162">
         <v>10000</v>
@@ -6987,10 +7003,10 @@
         <v>12</v>
       </c>
       <c r="B163" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C163" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="D163">
         <v>10000</v>
@@ -7016,10 +7032,10 @@
         <v>12</v>
       </c>
       <c r="B164" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C164" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D164">
         <v>10000</v>
@@ -7045,10 +7061,10 @@
         <v>12</v>
       </c>
       <c r="B165" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C165" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="D165">
         <v>10000</v>
@@ -7074,10 +7090,10 @@
         <v>12</v>
       </c>
       <c r="B166" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C166" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D166">
         <v>10000</v>
@@ -7103,10 +7119,10 @@
         <v>12</v>
       </c>
       <c r="B167" t="s">
+        <v>56</v>
+      </c>
+      <c r="C167" t="s">
         <v>38</v>
-      </c>
-      <c r="C167" t="s">
-        <v>16</v>
       </c>
       <c r="D167">
         <v>10000</v>
@@ -7132,10 +7148,10 @@
         <v>12</v>
       </c>
       <c r="B168" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="C168" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D168">
         <v>10000</v>
@@ -7161,10 +7177,10 @@
         <v>12</v>
       </c>
       <c r="B169" t="s">
+        <v>38</v>
+      </c>
+      <c r="C169" t="s">
         <v>16</v>
-      </c>
-      <c r="C169" t="s">
-        <v>38</v>
       </c>
       <c r="D169">
         <v>10000</v>
@@ -7190,10 +7206,10 @@
         <v>12</v>
       </c>
       <c r="B170" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="C170" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="D170">
         <v>10000</v>
@@ -7222,7 +7238,7 @@
         <v>16</v>
       </c>
       <c r="C171" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D171">
         <v>10000</v>
@@ -7251,7 +7267,7 @@
         <v>16</v>
       </c>
       <c r="C172" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="D172">
         <v>10000</v>
@@ -7277,10 +7293,10 @@
         <v>12</v>
       </c>
       <c r="B173" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="C173" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="D173">
         <v>10000</v>
@@ -7306,10 +7322,10 @@
         <v>12</v>
       </c>
       <c r="B174" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="C174" t="s">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="D174">
         <v>10000</v>
@@ -7335,7 +7351,7 @@
         <v>12</v>
       </c>
       <c r="B175" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C175" t="s">
         <v>16</v>
@@ -7364,10 +7380,10 @@
         <v>12</v>
       </c>
       <c r="B176" t="s">
+        <v>28</v>
+      </c>
+      <c r="C176" t="s">
         <v>42</v>
-      </c>
-      <c r="C176" t="s">
-        <v>28</v>
       </c>
       <c r="D176">
         <v>10000</v>
@@ -7396,7 +7412,7 @@
         <v>42</v>
       </c>
       <c r="C177" t="s">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="D177">
         <v>10000</v>
@@ -7425,7 +7441,7 @@
         <v>42</v>
       </c>
       <c r="C178" t="s">
-        <v>61</v>
+        <v>28</v>
       </c>
       <c r="D178">
         <v>10000</v>
@@ -7454,7 +7470,7 @@
         <v>42</v>
       </c>
       <c r="C179" t="s">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="D179">
         <v>10000</v>
@@ -7483,7 +7499,7 @@
         <v>42</v>
       </c>
       <c r="C180" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="D180">
         <v>10000</v>
@@ -7512,7 +7528,7 @@
         <v>42</v>
       </c>
       <c r="C181" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="D181">
         <v>10000</v>
@@ -7541,7 +7557,7 @@
         <v>42</v>
       </c>
       <c r="C182" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="D182">
         <v>10000</v>
@@ -7570,7 +7586,7 @@
         <v>42</v>
       </c>
       <c r="C183" t="s">
-        <v>63</v>
+        <v>30</v>
       </c>
       <c r="D183">
         <v>10000</v>
@@ -7596,10 +7612,10 @@
         <v>12</v>
       </c>
       <c r="B184" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="C184" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D184">
         <v>10000</v>
@@ -7625,10 +7641,10 @@
         <v>12</v>
       </c>
       <c r="B185" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="C185" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="D185">
         <v>10000</v>
@@ -7657,7 +7673,7 @@
         <v>60</v>
       </c>
       <c r="C186" t="s">
-        <v>64</v>
+        <v>42</v>
       </c>
       <c r="D186">
         <v>10000</v>
@@ -7686,7 +7702,7 @@
         <v>60</v>
       </c>
       <c r="C187" t="s">
-        <v>65</v>
+        <v>22</v>
       </c>
       <c r="D187">
         <v>10000</v>
@@ -7715,7 +7731,7 @@
         <v>60</v>
       </c>
       <c r="C188" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D188">
         <v>10000</v>
@@ -7741,10 +7757,10 @@
         <v>12</v>
       </c>
       <c r="B189" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="C189" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D189">
         <v>10000</v>
@@ -7770,10 +7786,10 @@
         <v>12</v>
       </c>
       <c r="B190" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="C190" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D190">
         <v>10000</v>
@@ -7802,7 +7818,7 @@
         <v>22</v>
       </c>
       <c r="C191" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D191">
         <v>10000</v>
@@ -7828,10 +7844,10 @@
         <v>12</v>
       </c>
       <c r="B192" t="s">
+        <v>22</v>
+      </c>
+      <c r="C192" t="s">
         <v>61</v>
-      </c>
-      <c r="C192" t="s">
-        <v>42</v>
       </c>
       <c r="D192">
         <v>10000</v>
@@ -7857,10 +7873,10 @@
         <v>12</v>
       </c>
       <c r="B193" t="s">
-        <v>61</v>
+        <v>22</v>
       </c>
       <c r="C193" t="s">
-        <v>22</v>
+        <v>64</v>
       </c>
       <c r="D193">
         <v>10000</v>
@@ -7889,7 +7905,7 @@
         <v>61</v>
       </c>
       <c r="C194" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="D194">
         <v>10000</v>
@@ -7915,7 +7931,7 @@
         <v>12</v>
       </c>
       <c r="B195" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C195" t="s">
         <v>22</v>
@@ -7944,10 +7960,10 @@
         <v>12</v>
       </c>
       <c r="B196" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C196" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D196">
         <v>10000</v>
@@ -7973,10 +7989,10 @@
         <v>12</v>
       </c>
       <c r="B197" t="s">
-        <v>24</v>
+        <v>64</v>
       </c>
       <c r="C197" t="s">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="D197">
         <v>10000</v>
@@ -8002,10 +8018,10 @@
         <v>12</v>
       </c>
       <c r="B198" t="s">
+        <v>64</v>
+      </c>
+      <c r="C198" t="s">
         <v>24</v>
-      </c>
-      <c r="C198" t="s">
-        <v>66</v>
       </c>
       <c r="D198">
         <v>10000</v>
@@ -8031,10 +8047,10 @@
         <v>12</v>
       </c>
       <c r="B199" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C199" t="s">
-        <v>16</v>
+        <v>64</v>
       </c>
       <c r="D199">
         <v>10000</v>
@@ -8060,10 +8076,10 @@
         <v>12</v>
       </c>
       <c r="B200" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C200" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D200">
         <v>10000</v>
@@ -8092,7 +8108,7 @@
         <v>18</v>
       </c>
       <c r="C201" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="D201">
         <v>10000</v>
@@ -8118,10 +8134,10 @@
         <v>12</v>
       </c>
       <c r="B202" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="C202" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="D202">
         <v>10000</v>
@@ -8147,10 +8163,10 @@
         <v>12</v>
       </c>
       <c r="B203" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="C203" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D203">
         <v>10000</v>
@@ -8176,7 +8192,7 @@
         <v>12</v>
       </c>
       <c r="B204" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="C204" t="s">
         <v>42</v>
@@ -8205,10 +8221,10 @@
         <v>12</v>
       </c>
       <c r="B205" t="s">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="C205" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D205">
         <v>10000</v>
@@ -8237,7 +8253,7 @@
         <v>62</v>
       </c>
       <c r="C206" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="D206">
         <v>10000</v>
@@ -8263,10 +8279,10 @@
         <v>12</v>
       </c>
       <c r="B207" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C207" t="s">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="D207">
         <v>10000</v>
@@ -8292,10 +8308,10 @@
         <v>12</v>
       </c>
       <c r="B208" t="s">
+        <v>62</v>
+      </c>
+      <c r="C208" t="s">
         <v>65</v>
-      </c>
-      <c r="C208" t="s">
-        <v>62</v>
       </c>
       <c r="D208">
         <v>10000</v>
@@ -8324,7 +8340,7 @@
         <v>65</v>
       </c>
       <c r="C209" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D209">
         <v>10000</v>
@@ -8353,7 +8369,7 @@
         <v>65</v>
       </c>
       <c r="C210" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D210">
         <v>10000</v>
@@ -8379,10 +8395,10 @@
         <v>12</v>
       </c>
       <c r="B211" t="s">
+        <v>65</v>
+      </c>
+      <c r="C211" t="s">
         <v>66</v>
-      </c>
-      <c r="C211" t="s">
-        <v>24</v>
       </c>
       <c r="D211">
         <v>10000</v>
@@ -8408,10 +8424,10 @@
         <v>12</v>
       </c>
       <c r="B212" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C212" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="D212">
         <v>10000</v>
@@ -8440,7 +8456,7 @@
         <v>66</v>
       </c>
       <c r="C213" t="s">
-        <v>67</v>
+        <v>24</v>
       </c>
       <c r="D213">
         <v>10000</v>
@@ -8469,7 +8485,7 @@
         <v>66</v>
       </c>
       <c r="C214" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="D214">
         <v>10000</v>
@@ -8495,10 +8511,10 @@
         <v>12</v>
       </c>
       <c r="B215" t="s">
+        <v>66</v>
+      </c>
+      <c r="C215" t="s">
         <v>67</v>
-      </c>
-      <c r="C215" t="s">
-        <v>68</v>
       </c>
       <c r="D215">
         <v>10000</v>
@@ -8524,10 +8540,10 @@
         <v>12</v>
       </c>
       <c r="B216" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C216" t="s">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="D216">
         <v>10000</v>
@@ -8553,10 +8569,10 @@
         <v>12</v>
       </c>
       <c r="B217" t="s">
+        <v>67</v>
+      </c>
+      <c r="C217" t="s">
         <v>68</v>
-      </c>
-      <c r="C217" t="s">
-        <v>67</v>
       </c>
       <c r="D217">
         <v>10000</v>
@@ -8582,10 +8598,10 @@
         <v>12</v>
       </c>
       <c r="B218" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C218" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="D218">
         <v>10000</v>
@@ -8614,7 +8630,7 @@
         <v>68</v>
       </c>
       <c r="C219" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="D219">
         <v>10000</v>
@@ -8643,7 +8659,7 @@
         <v>68</v>
       </c>
       <c r="C220" t="s">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="D220">
         <v>10000</v>
@@ -8672,7 +8688,7 @@
         <v>68</v>
       </c>
       <c r="C221" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="D221">
         <v>10000</v>
@@ -8698,10 +8714,10 @@
         <v>12</v>
       </c>
       <c r="B222" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="C222" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D222">
         <v>10000</v>
@@ -8727,10 +8743,10 @@
         <v>12</v>
       </c>
       <c r="B223" t="s">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="C223" t="s">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="D223">
         <v>10000</v>
@@ -8756,7 +8772,7 @@
         <v>12</v>
       </c>
       <c r="B224" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="C224" t="s">
         <v>68</v>
@@ -8788,7 +8804,7 @@
         <v>51</v>
       </c>
       <c r="C225" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="D225">
         <v>10000</v>
@@ -8817,7 +8833,7 @@
         <v>51</v>
       </c>
       <c r="C226" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D226">
         <v>10000</v>
@@ -8843,10 +8859,10 @@
         <v>12</v>
       </c>
       <c r="B227" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="C227" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="D227">
         <v>10000</v>
@@ -8872,10 +8888,10 @@
         <v>12</v>
       </c>
       <c r="B228" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="C228" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="D228">
         <v>10000</v>
@@ -8901,10 +8917,10 @@
         <v>12</v>
       </c>
       <c r="B229" t="s">
+        <v>26</v>
+      </c>
+      <c r="C229" t="s">
         <v>72</v>
-      </c>
-      <c r="C229" t="s">
-        <v>26</v>
       </c>
       <c r="D229">
         <v>10000</v>
@@ -8930,7 +8946,7 @@
         <v>12</v>
       </c>
       <c r="B230" t="s">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="C230" t="s">
         <v>53</v>
@@ -8959,10 +8975,10 @@
         <v>12</v>
       </c>
       <c r="B231" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="C231" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D231">
         <v>10000</v>
@@ -8988,10 +9004,10 @@
         <v>12</v>
       </c>
       <c r="B232" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="C232" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="D232">
         <v>10000</v>
@@ -9017,10 +9033,10 @@
         <v>12</v>
       </c>
       <c r="B233" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C233" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="D233">
         <v>10000</v>
@@ -9046,10 +9062,10 @@
         <v>12</v>
       </c>
       <c r="B234" t="s">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="C234" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D234">
         <v>10000</v>
@@ -9075,10 +9091,10 @@
         <v>12</v>
       </c>
       <c r="B235" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="C235" t="s">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="D235">
         <v>10000</v>
@@ -9107,7 +9123,7 @@
         <v>58</v>
       </c>
       <c r="C236" t="s">
-        <v>66</v>
+        <v>30</v>
       </c>
       <c r="D236">
         <v>10000</v>
@@ -9136,7 +9152,7 @@
         <v>58</v>
       </c>
       <c r="C237" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="D237">
         <v>10000</v>
@@ -9162,10 +9178,10 @@
         <v>12</v>
       </c>
       <c r="B238" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="C238" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="D238">
         <v>10000</v>
@@ -9191,10 +9207,10 @@
         <v>12</v>
       </c>
       <c r="B239" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C239" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="D239">
         <v>10000</v>
@@ -9220,10 +9236,10 @@
         <v>12</v>
       </c>
       <c r="B240" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="C240" t="s">
-        <v>72</v>
+        <v>51</v>
       </c>
       <c r="D240">
         <v>10000</v>
@@ -9252,7 +9268,7 @@
         <v>53</v>
       </c>
       <c r="C241" t="s">
-        <v>73</v>
+        <v>42</v>
       </c>
       <c r="D241">
         <v>10000</v>
@@ -9278,10 +9294,10 @@
         <v>12</v>
       </c>
       <c r="B242" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="C242" t="s">
-        <v>22</v>
+        <v>72</v>
       </c>
       <c r="D242">
         <v>10000</v>
@@ -9307,10 +9323,10 @@
         <v>12</v>
       </c>
       <c r="B243" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="C243" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="D243">
         <v>10000</v>
@@ -9336,10 +9352,10 @@
         <v>12</v>
       </c>
       <c r="B244" t="s">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="C244" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D244">
         <v>10000</v>
@@ -9365,10 +9381,10 @@
         <v>12</v>
       </c>
       <c r="B245" t="s">
-        <v>77</v>
+        <v>36</v>
       </c>
       <c r="C245" t="s">
-        <v>34</v>
+        <v>68</v>
       </c>
       <c r="D245">
         <v>10000</v>
@@ -9394,10 +9410,10 @@
         <v>12</v>
       </c>
       <c r="B246" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="C246" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D246">
         <v>10000</v>
@@ -9423,10 +9439,10 @@
         <v>12</v>
       </c>
       <c r="B247" t="s">
-        <v>45</v>
+        <v>77</v>
       </c>
       <c r="C247" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="D247">
         <v>10000</v>
@@ -9452,10 +9468,10 @@
         <v>12</v>
       </c>
       <c r="B248" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="C248" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="D248">
         <v>10000</v>
@@ -9481,10 +9497,10 @@
         <v>12</v>
       </c>
       <c r="B249" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="C249" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D249">
         <v>10000</v>
@@ -9510,10 +9526,10 @@
         <v>12</v>
       </c>
       <c r="B250" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="C250" t="s">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="D250">
         <v>10000</v>
@@ -9539,10 +9555,10 @@
         <v>12</v>
       </c>
       <c r="B251" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C251" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="D251">
         <v>10000</v>
@@ -9568,10 +9584,10 @@
         <v>12</v>
       </c>
       <c r="B252" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="C252" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="D252">
         <v>10000</v>
@@ -9597,10 +9613,10 @@
         <v>12</v>
       </c>
       <c r="B253" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="C253" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D253">
         <v>10000</v>
@@ -9626,10 +9642,10 @@
         <v>12</v>
       </c>
       <c r="B254" t="s">
-        <v>48</v>
+        <v>67</v>
       </c>
       <c r="C254" t="s">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="D254">
         <v>10000</v>
@@ -9655,10 +9671,10 @@
         <v>12</v>
       </c>
       <c r="B255" t="s">
-        <v>48</v>
+        <v>82</v>
       </c>
       <c r="C255" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D255">
         <v>10000</v>
@@ -9687,7 +9703,7 @@
         <v>48</v>
       </c>
       <c r="C256" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="D256">
         <v>10000</v>
@@ -9716,7 +9732,7 @@
         <v>48</v>
       </c>
       <c r="C257" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="D257">
         <v>10000</v>
@@ -9745,7 +9761,7 @@
         <v>48</v>
       </c>
       <c r="C258" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="D258">
         <v>10000</v>
@@ -9771,10 +9787,10 @@
         <v>12</v>
       </c>
       <c r="B259" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="C259" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D259">
         <v>10000</v>
@@ -9800,10 +9816,10 @@
         <v>12</v>
       </c>
       <c r="B260" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="C260" t="s">
-        <v>74</v>
+        <v>38</v>
       </c>
       <c r="D260">
         <v>10000</v>
@@ -9829,10 +9845,10 @@
         <v>12</v>
       </c>
       <c r="B261" t="s">
-        <v>82</v>
+        <v>38</v>
       </c>
       <c r="C261" t="s">
-        <v>77</v>
+        <v>28</v>
       </c>
       <c r="D261">
         <v>10000</v>
@@ -9858,10 +9874,10 @@
         <v>12</v>
       </c>
       <c r="B262" t="s">
-        <v>82</v>
+        <v>20</v>
       </c>
       <c r="C262" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="D262">
         <v>10000</v>
@@ -9887,10 +9903,10 @@
         <v>12</v>
       </c>
       <c r="B263" t="s">
-        <v>40</v>
+        <v>82</v>
       </c>
       <c r="C263" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D263">
         <v>10000</v>
@@ -9916,10 +9932,10 @@
         <v>12</v>
       </c>
       <c r="B264" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C264" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="D264">
         <v>10000</v>
@@ -9928,7 +9944,7 @@
         <v>10000</v>
       </c>
       <c r="F264">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G264">
         <v>10000000</v>
@@ -9945,10 +9961,10 @@
         <v>12</v>
       </c>
       <c r="B265" t="s">
-        <v>81</v>
+        <v>40</v>
       </c>
       <c r="C265" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D265">
         <v>10000</v>
@@ -9957,7 +9973,7 @@
         <v>10000</v>
       </c>
       <c r="F265">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G265">
         <v>10000000</v>
@@ -9974,10 +9990,10 @@
         <v>12</v>
       </c>
       <c r="B266" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C266" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="D266">
         <v>10000</v>
@@ -10003,10 +10019,10 @@
         <v>12</v>
       </c>
       <c r="B267" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C267" t="s">
-        <v>16</v>
+        <v>82</v>
       </c>
       <c r="D267">
         <v>10000</v>
@@ -10032,10 +10048,10 @@
         <v>12</v>
       </c>
       <c r="B268" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C268" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="D268">
         <v>10000</v>
@@ -10061,10 +10077,10 @@
         <v>12</v>
       </c>
       <c r="B269" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C269" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D269">
         <v>10000</v>
@@ -10090,10 +10106,10 @@
         <v>12</v>
       </c>
       <c r="B270" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C270" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D270">
         <v>10000</v>
@@ -10119,10 +10135,10 @@
         <v>12</v>
       </c>
       <c r="B271" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C271" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="D271">
         <v>10000</v>
@@ -10148,10 +10164,10 @@
         <v>12</v>
       </c>
       <c r="B272" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C272" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="D272">
         <v>10000</v>
@@ -10177,10 +10193,10 @@
         <v>12</v>
       </c>
       <c r="B273" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C273" t="s">
-        <v>66</v>
+        <v>18</v>
       </c>
       <c r="D273">
         <v>10000</v>
@@ -10206,10 +10222,10 @@
         <v>12</v>
       </c>
       <c r="B274" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C274" t="s">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="D274">
         <v>10000</v>
@@ -10235,10 +10251,10 @@
         <v>12</v>
       </c>
       <c r="B275" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C275" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D275">
         <v>10000</v>
@@ -10264,10 +10280,10 @@
         <v>12</v>
       </c>
       <c r="B276" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C276" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="D276">
         <v>10000</v>
@@ -10293,10 +10309,10 @@
         <v>12</v>
       </c>
       <c r="B277" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C277" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D277">
         <v>10000</v>
@@ -10322,10 +10338,10 @@
         <v>12</v>
       </c>
       <c r="B278" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C278" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="D278">
         <v>10000</v>
@@ -10351,10 +10367,10 @@
         <v>12</v>
       </c>
       <c r="B279" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C279" t="s">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="D279">
         <v>10000</v>
@@ -10380,10 +10396,10 @@
         <v>12</v>
       </c>
       <c r="B280" t="s">
-        <v>53</v>
+        <v>95</v>
       </c>
       <c r="C280" t="s">
-        <v>75</v>
+        <v>36</v>
       </c>
       <c r="D280">
         <v>10000</v>
@@ -10392,7 +10408,7 @@
         <v>10000</v>
       </c>
       <c r="F280">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="G280">
         <v>10000000</v>
@@ -10409,27 +10425,143 @@
         <v>12</v>
       </c>
       <c r="B281" t="s">
+        <v>96</v>
+      </c>
+      <c r="C281" t="s">
+        <v>34</v>
+      </c>
+      <c r="D281">
+        <v>10000</v>
+      </c>
+      <c r="E281">
+        <v>10000</v>
+      </c>
+      <c r="F281">
+        <v>100</v>
+      </c>
+      <c r="G281">
+        <v>10000000</v>
+      </c>
+      <c r="H281">
+        <v>1000</v>
+      </c>
+      <c r="I281">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="282" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A282" t="s">
+        <v>12</v>
+      </c>
+      <c r="B282" t="s">
+        <v>53</v>
+      </c>
+      <c r="C282" t="s">
         <v>75</v>
       </c>
-      <c r="C281" t="s">
+      <c r="D282">
+        <v>10000</v>
+      </c>
+      <c r="E282">
+        <v>10000</v>
+      </c>
+      <c r="F282">
+        <v>1</v>
+      </c>
+      <c r="G282">
+        <v>10000000</v>
+      </c>
+      <c r="H282">
+        <v>1000</v>
+      </c>
+      <c r="I282">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="283" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A283" t="s">
+        <v>12</v>
+      </c>
+      <c r="B283" t="s">
+        <v>75</v>
+      </c>
+      <c r="C283" t="s">
         <v>30</v>
       </c>
-      <c r="D281">
-        <v>10000</v>
-      </c>
-      <c r="E281">
-        <v>10000</v>
-      </c>
-      <c r="F281">
-        <v>1</v>
-      </c>
-      <c r="G281">
-        <v>10000000</v>
-      </c>
-      <c r="H281">
-        <v>1000</v>
-      </c>
-      <c r="I281">
+      <c r="D283">
+        <v>10000</v>
+      </c>
+      <c r="E283">
+        <v>10000</v>
+      </c>
+      <c r="F283">
+        <v>1</v>
+      </c>
+      <c r="G283">
+        <v>10000000</v>
+      </c>
+      <c r="H283">
+        <v>1000</v>
+      </c>
+      <c r="I283">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="284" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A284" t="s">
+        <v>12</v>
+      </c>
+      <c r="B284" t="s">
+        <v>97</v>
+      </c>
+      <c r="C284" t="s">
+        <v>72</v>
+      </c>
+      <c r="D284">
+        <v>10000</v>
+      </c>
+      <c r="E284">
+        <v>10000</v>
+      </c>
+      <c r="F284">
+        <v>100</v>
+      </c>
+      <c r="G284">
+        <v>10000000</v>
+      </c>
+      <c r="H284">
+        <v>1000</v>
+      </c>
+      <c r="I284">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="285" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A285" t="s">
+        <v>12</v>
+      </c>
+      <c r="B285" t="s">
+        <v>72</v>
+      </c>
+      <c r="C285" t="s">
+        <v>97</v>
+      </c>
+      <c r="D285">
+        <v>10000</v>
+      </c>
+      <c r="E285">
+        <v>10000</v>
+      </c>
+      <c r="F285">
+        <v>100</v>
+      </c>
+      <c r="G285">
+        <v>10000000</v>
+      </c>
+      <c r="H285">
+        <v>1000</v>
+      </c>
+      <c r="I285">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add missing connections to BASE case
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/data_case_russia_BASE.xlsx
+++ b/01_data/01_input_data/02_processed/data_case_russia_BASE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C7CE7E8-146D-4101-B7C4-1C8222EA1E9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7F9548E-9359-4B54-9505-316583751CCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="4" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1574" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1586" uniqueCount="98">
   <si>
     <t>Commodities</t>
   </si>
@@ -1151,7 +1151,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA366CBE-E84C-4E05-9B58-54F3A95EEAB7}">
-  <dimension ref="A1:B142"/>
+  <dimension ref="A1:B148"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -2288,6 +2288,54 @@
       </c>
       <c r="B142" t="s">
         <v>32</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A143" t="s">
+        <v>69</v>
+      </c>
+      <c r="B143" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A144" t="s">
+        <v>56</v>
+      </c>
+      <c r="B144" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A145" t="s">
+        <v>73</v>
+      </c>
+      <c r="B145" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A146" t="s">
+        <v>66</v>
+      </c>
+      <c r="B146" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A147" t="s">
+        <v>71</v>
+      </c>
+      <c r="B147" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A148" t="s">
+        <v>94</v>
+      </c>
+      <c r="B148" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add LNG import-export countries/regions other than in Europe
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/data_case_russia_BASE.xlsx
+++ b/01_data/01_input_data/02_processed/data_case_russia_BASE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C173888F-F51F-4B80-A114-3EF0BCFD2697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D89C1AB0-EB9C-4A68-81BA-2451B45FE05D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1588" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1930" uniqueCount="134">
   <si>
     <t>Commodities</t>
   </si>
@@ -334,6 +334,114 @@
   </si>
   <si>
     <t>EL_Prod</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>USA_Prod</t>
+  </si>
+  <si>
+    <t>USA_LNG</t>
+  </si>
+  <si>
+    <t>NA_prod</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>NA_LNG</t>
+  </si>
+  <si>
+    <t>SA</t>
+  </si>
+  <si>
+    <t>SA_Prod</t>
+  </si>
+  <si>
+    <t>SA_LNG</t>
+  </si>
+  <si>
+    <t>TT</t>
+  </si>
+  <si>
+    <t>TT_Prod</t>
+  </si>
+  <si>
+    <t>TT_LNG</t>
+  </si>
+  <si>
+    <t>ME</t>
+  </si>
+  <si>
+    <t>ME_Prod</t>
+  </si>
+  <si>
+    <t>ME_LNG</t>
+  </si>
+  <si>
+    <t>QA</t>
+  </si>
+  <si>
+    <t>QA_Prod</t>
+  </si>
+  <si>
+    <t>QA_LNG</t>
+  </si>
+  <si>
+    <t>AF</t>
+  </si>
+  <si>
+    <t>AF_Prod</t>
+  </si>
+  <si>
+    <t>AF_LNG</t>
+  </si>
+  <si>
+    <t>AU</t>
+  </si>
+  <si>
+    <t>AU_Prod</t>
+  </si>
+  <si>
+    <t>AU_LNG</t>
+  </si>
+  <si>
+    <t>CN</t>
+  </si>
+  <si>
+    <t>CN_Prod</t>
+  </si>
+  <si>
+    <t>CN_LNG</t>
+  </si>
+  <si>
+    <t>JS</t>
+  </si>
+  <si>
+    <t>JS_Prod</t>
+  </si>
+  <si>
+    <t>JS_LNG</t>
+  </si>
+  <si>
+    <t>IN</t>
+  </si>
+  <si>
+    <t>IN_Prod</t>
+  </si>
+  <si>
+    <t>IN_LNG</t>
+  </si>
+  <si>
+    <t>AS</t>
+  </si>
+  <si>
+    <t>AS_Prod</t>
+  </si>
+  <si>
+    <t>AS_LNG</t>
   </si>
 </sst>
 </file>
@@ -691,7 +799,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B0CB446-BDDD-415D-AF22-2CEB1FE45CA5}">
-  <dimension ref="A1:A85"/>
+  <dimension ref="A1:A121"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -1117,6 +1225,186 @@
     <row r="85" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>68</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A111" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A114" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A115" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A120" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A121" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -1151,7 +1439,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA366CBE-E84C-4E05-9B58-54F3A95EEAB7}">
-  <dimension ref="A1:B149"/>
+  <dimension ref="A1:B164"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -2344,6 +2632,126 @@
       </c>
       <c r="B149" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A150" t="s">
+        <v>100</v>
+      </c>
+      <c r="B150" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A151" t="s">
+        <v>99</v>
+      </c>
+      <c r="B151" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A152" t="s">
+        <v>98</v>
+      </c>
+      <c r="B152" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A153" t="s">
+        <v>100</v>
+      </c>
+      <c r="B153" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A154" t="s">
+        <v>100</v>
+      </c>
+      <c r="B154" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A155" t="s">
+        <v>100</v>
+      </c>
+      <c r="B155" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A156" t="s">
+        <v>100</v>
+      </c>
+      <c r="B156" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A157" t="s">
+        <v>100</v>
+      </c>
+      <c r="B157" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A158" t="s">
+        <v>100</v>
+      </c>
+      <c r="B158" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A159" t="s">
+        <v>100</v>
+      </c>
+      <c r="B159" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A160" t="s">
+        <v>100</v>
+      </c>
+      <c r="B160" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A161" t="s">
+        <v>100</v>
+      </c>
+      <c r="B161" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A162" t="s">
+        <v>100</v>
+      </c>
+      <c r="B162" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A163" t="s">
+        <v>100</v>
+      </c>
+      <c r="B163" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A164" t="s">
+        <v>100</v>
+      </c>
+      <c r="B164" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -2353,7 +2761,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C781A78E-EFEC-4F2E-A496-3B44BD173FD3}">
-  <dimension ref="A1:I285"/>
+  <dimension ref="A1:I329"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -10618,6 +11026,1282 @@
         <v>1000</v>
       </c>
       <c r="I285">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="286" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A286" t="s">
+        <v>11</v>
+      </c>
+      <c r="B286" t="s">
+        <v>100</v>
+      </c>
+      <c r="C286" t="s">
+        <v>31</v>
+      </c>
+      <c r="D286">
+        <v>10000</v>
+      </c>
+      <c r="E286">
+        <v>10000</v>
+      </c>
+      <c r="F286">
+        <v>20</v>
+      </c>
+      <c r="G286">
+        <v>10000000</v>
+      </c>
+      <c r="H286">
+        <v>0</v>
+      </c>
+      <c r="I286">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="287" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A287" t="s">
+        <v>11</v>
+      </c>
+      <c r="B287" t="s">
+        <v>99</v>
+      </c>
+      <c r="C287" t="s">
+        <v>98</v>
+      </c>
+      <c r="D287">
+        <v>10000</v>
+      </c>
+      <c r="E287">
+        <v>10000</v>
+      </c>
+      <c r="F287">
+        <v>100</v>
+      </c>
+      <c r="G287">
+        <v>10000000</v>
+      </c>
+      <c r="H287">
+        <v>0</v>
+      </c>
+      <c r="I287">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="288" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A288" t="s">
+        <v>11</v>
+      </c>
+      <c r="B288" t="s">
+        <v>98</v>
+      </c>
+      <c r="C288" t="s">
+        <v>100</v>
+      </c>
+      <c r="D288">
+        <v>10000</v>
+      </c>
+      <c r="E288">
+        <v>10000</v>
+      </c>
+      <c r="F288">
+        <v>100</v>
+      </c>
+      <c r="G288">
+        <v>10000000</v>
+      </c>
+      <c r="H288">
+        <v>0</v>
+      </c>
+      <c r="I288">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="289" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A289" t="s">
+        <v>12</v>
+      </c>
+      <c r="B289" t="s">
+        <v>100</v>
+      </c>
+      <c r="C289" t="s">
+        <v>31</v>
+      </c>
+      <c r="D289">
+        <v>10000</v>
+      </c>
+      <c r="E289">
+        <v>10000</v>
+      </c>
+      <c r="F289">
+        <v>100</v>
+      </c>
+      <c r="G289">
+        <v>10000000</v>
+      </c>
+      <c r="H289">
+        <v>1000</v>
+      </c>
+      <c r="I289">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="290" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A290" t="s">
+        <v>12</v>
+      </c>
+      <c r="B290" t="s">
+        <v>99</v>
+      </c>
+      <c r="C290" t="s">
+        <v>98</v>
+      </c>
+      <c r="D290">
+        <v>10000</v>
+      </c>
+      <c r="E290">
+        <v>10000</v>
+      </c>
+      <c r="F290">
+        <v>100</v>
+      </c>
+      <c r="G290">
+        <v>10000000</v>
+      </c>
+      <c r="H290">
+        <v>1000</v>
+      </c>
+      <c r="I290">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="291" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A291" t="s">
+        <v>12</v>
+      </c>
+      <c r="B291" t="s">
+        <v>98</v>
+      </c>
+      <c r="C291" t="s">
+        <v>100</v>
+      </c>
+      <c r="D291">
+        <v>10000</v>
+      </c>
+      <c r="E291">
+        <v>10000</v>
+      </c>
+      <c r="F291">
+        <v>100</v>
+      </c>
+      <c r="G291">
+        <v>10000000</v>
+      </c>
+      <c r="H291">
+        <v>1000</v>
+      </c>
+      <c r="I291">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="292" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A292" t="s">
+        <v>11</v>
+      </c>
+      <c r="B292" t="s">
+        <v>69</v>
+      </c>
+      <c r="C292" t="s">
+        <v>56</v>
+      </c>
+      <c r="D292">
+        <v>10000</v>
+      </c>
+      <c r="E292">
+        <v>10000</v>
+      </c>
+      <c r="F292">
+        <v>100</v>
+      </c>
+      <c r="G292">
+        <v>10000000</v>
+      </c>
+      <c r="H292">
+        <v>0</v>
+      </c>
+      <c r="I292">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="293" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A293" t="s">
+        <v>11</v>
+      </c>
+      <c r="B293" t="s">
+        <v>56</v>
+      </c>
+      <c r="C293" t="s">
+        <v>69</v>
+      </c>
+      <c r="D293">
+        <v>10000</v>
+      </c>
+      <c r="E293">
+        <v>10000</v>
+      </c>
+      <c r="F293">
+        <v>100</v>
+      </c>
+      <c r="G293">
+        <v>10000000</v>
+      </c>
+      <c r="H293">
+        <v>0</v>
+      </c>
+      <c r="I293">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="294" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A294" t="s">
+        <v>11</v>
+      </c>
+      <c r="B294" t="s">
+        <v>73</v>
+      </c>
+      <c r="C294" t="s">
+        <v>56</v>
+      </c>
+      <c r="D294">
+        <v>10000</v>
+      </c>
+      <c r="E294">
+        <v>10000</v>
+      </c>
+      <c r="F294">
+        <v>100</v>
+      </c>
+      <c r="G294">
+        <v>10000000</v>
+      </c>
+      <c r="H294">
+        <v>0</v>
+      </c>
+      <c r="I294">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="295" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A295" t="s">
+        <v>11</v>
+      </c>
+      <c r="B295" t="s">
+        <v>16</v>
+      </c>
+      <c r="C295" t="s">
+        <v>61</v>
+      </c>
+      <c r="D295">
+        <v>10000</v>
+      </c>
+      <c r="E295">
+        <v>10000</v>
+      </c>
+      <c r="F295">
+        <v>100</v>
+      </c>
+      <c r="G295">
+        <v>10000000</v>
+      </c>
+      <c r="H295">
+        <v>0</v>
+      </c>
+      <c r="I295">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="296" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A296" t="s">
+        <v>11</v>
+      </c>
+      <c r="B296" t="s">
+        <v>71</v>
+      </c>
+      <c r="C296" t="s">
+        <v>94</v>
+      </c>
+      <c r="D296">
+        <v>10000</v>
+      </c>
+      <c r="E296">
+        <v>10000</v>
+      </c>
+      <c r="F296">
+        <v>100</v>
+      </c>
+      <c r="G296">
+        <v>10000000</v>
+      </c>
+      <c r="H296">
+        <v>0</v>
+      </c>
+      <c r="I296">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="297" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A297" t="s">
+        <v>11</v>
+      </c>
+      <c r="B297" t="s">
+        <v>94</v>
+      </c>
+      <c r="C297" t="s">
+        <v>71</v>
+      </c>
+      <c r="D297">
+        <v>10000</v>
+      </c>
+      <c r="E297">
+        <v>10000</v>
+      </c>
+      <c r="F297">
+        <v>100</v>
+      </c>
+      <c r="G297">
+        <v>10000000</v>
+      </c>
+      <c r="H297">
+        <v>0</v>
+      </c>
+      <c r="I297">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="298" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A298" t="s">
+        <v>11</v>
+      </c>
+      <c r="B298" t="s">
+        <v>51</v>
+      </c>
+      <c r="C298" t="s">
+        <v>34</v>
+      </c>
+      <c r="D298">
+        <v>10000</v>
+      </c>
+      <c r="E298">
+        <v>10000</v>
+      </c>
+      <c r="F298">
+        <v>100</v>
+      </c>
+      <c r="G298">
+        <v>10000000</v>
+      </c>
+      <c r="H298">
+        <v>0</v>
+      </c>
+      <c r="I298">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="299" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A299" t="s">
+        <v>12</v>
+      </c>
+      <c r="B299" t="s">
+        <v>69</v>
+      </c>
+      <c r="C299" t="s">
+        <v>56</v>
+      </c>
+      <c r="D299">
+        <v>10000</v>
+      </c>
+      <c r="E299">
+        <v>10000</v>
+      </c>
+      <c r="F299">
+        <v>100</v>
+      </c>
+      <c r="G299">
+        <v>10000000</v>
+      </c>
+      <c r="H299">
+        <v>1000</v>
+      </c>
+      <c r="I299">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="300" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A300" t="s">
+        <v>12</v>
+      </c>
+      <c r="B300" t="s">
+        <v>56</v>
+      </c>
+      <c r="C300" t="s">
+        <v>69</v>
+      </c>
+      <c r="D300">
+        <v>10000</v>
+      </c>
+      <c r="E300">
+        <v>10000</v>
+      </c>
+      <c r="F300">
+        <v>100</v>
+      </c>
+      <c r="G300">
+        <v>10000000</v>
+      </c>
+      <c r="H300">
+        <v>1000</v>
+      </c>
+      <c r="I300">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="301" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A301" t="s">
+        <v>12</v>
+      </c>
+      <c r="B301" t="s">
+        <v>73</v>
+      </c>
+      <c r="C301" t="s">
+        <v>56</v>
+      </c>
+      <c r="D301">
+        <v>10000</v>
+      </c>
+      <c r="E301">
+        <v>10000</v>
+      </c>
+      <c r="F301">
+        <v>100</v>
+      </c>
+      <c r="G301">
+        <v>10000000</v>
+      </c>
+      <c r="H301">
+        <v>1000</v>
+      </c>
+      <c r="I301">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="302" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A302" t="s">
+        <v>12</v>
+      </c>
+      <c r="B302" t="s">
+        <v>16</v>
+      </c>
+      <c r="C302" t="s">
+        <v>61</v>
+      </c>
+      <c r="D302">
+        <v>10000</v>
+      </c>
+      <c r="E302">
+        <v>10000</v>
+      </c>
+      <c r="F302">
+        <v>100</v>
+      </c>
+      <c r="G302">
+        <v>10000000</v>
+      </c>
+      <c r="H302">
+        <v>1000</v>
+      </c>
+      <c r="I302">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="303" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A303" t="s">
+        <v>12</v>
+      </c>
+      <c r="B303" t="s">
+        <v>71</v>
+      </c>
+      <c r="C303" t="s">
+        <v>94</v>
+      </c>
+      <c r="D303">
+        <v>10000</v>
+      </c>
+      <c r="E303">
+        <v>10000</v>
+      </c>
+      <c r="F303">
+        <v>100</v>
+      </c>
+      <c r="G303">
+        <v>10000000</v>
+      </c>
+      <c r="H303">
+        <v>1000</v>
+      </c>
+      <c r="I303">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="304" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A304" t="s">
+        <v>12</v>
+      </c>
+      <c r="B304" t="s">
+        <v>94</v>
+      </c>
+      <c r="C304" t="s">
+        <v>71</v>
+      </c>
+      <c r="D304">
+        <v>10000</v>
+      </c>
+      <c r="E304">
+        <v>10000</v>
+      </c>
+      <c r="F304">
+        <v>100</v>
+      </c>
+      <c r="G304">
+        <v>10000000</v>
+      </c>
+      <c r="H304">
+        <v>1000</v>
+      </c>
+      <c r="I304">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="305" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A305" t="s">
+        <v>12</v>
+      </c>
+      <c r="B305" t="s">
+        <v>51</v>
+      </c>
+      <c r="C305" t="s">
+        <v>34</v>
+      </c>
+      <c r="D305">
+        <v>10000</v>
+      </c>
+      <c r="E305">
+        <v>10000</v>
+      </c>
+      <c r="F305">
+        <v>100</v>
+      </c>
+      <c r="G305">
+        <v>10000000</v>
+      </c>
+      <c r="H305">
+        <v>1000</v>
+      </c>
+      <c r="I305">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="306" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A306" t="s">
+        <v>11</v>
+      </c>
+      <c r="B306" t="s">
+        <v>100</v>
+      </c>
+      <c r="C306" t="s">
+        <v>15</v>
+      </c>
+      <c r="D306">
+        <v>10000</v>
+      </c>
+      <c r="E306">
+        <v>10000</v>
+      </c>
+      <c r="F306">
+        <v>20</v>
+      </c>
+      <c r="G306">
+        <v>10000000</v>
+      </c>
+      <c r="H306">
+        <v>0</v>
+      </c>
+      <c r="I306">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="307" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A307" t="s">
+        <v>11</v>
+      </c>
+      <c r="B307" t="s">
+        <v>100</v>
+      </c>
+      <c r="C307" t="s">
+        <v>17</v>
+      </c>
+      <c r="D307">
+        <v>10000</v>
+      </c>
+      <c r="E307">
+        <v>10000</v>
+      </c>
+      <c r="F307">
+        <v>20</v>
+      </c>
+      <c r="G307">
+        <v>10000000</v>
+      </c>
+      <c r="H307">
+        <v>0</v>
+      </c>
+      <c r="I307">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="308" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A308" t="s">
+        <v>11</v>
+      </c>
+      <c r="B308" t="s">
+        <v>100</v>
+      </c>
+      <c r="C308" t="s">
+        <v>95</v>
+      </c>
+      <c r="D308">
+        <v>10000</v>
+      </c>
+      <c r="E308">
+        <v>10000</v>
+      </c>
+      <c r="F308">
+        <v>20</v>
+      </c>
+      <c r="G308">
+        <v>10000000</v>
+      </c>
+      <c r="H308">
+        <v>0</v>
+      </c>
+      <c r="I308">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="309" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A309" t="s">
+        <v>11</v>
+      </c>
+      <c r="B309" t="s">
+        <v>100</v>
+      </c>
+      <c r="C309" t="s">
+        <v>19</v>
+      </c>
+      <c r="D309">
+        <v>10000</v>
+      </c>
+      <c r="E309">
+        <v>10000</v>
+      </c>
+      <c r="F309">
+        <v>20</v>
+      </c>
+      <c r="G309">
+        <v>10000000</v>
+      </c>
+      <c r="H309">
+        <v>0</v>
+      </c>
+      <c r="I309">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="310" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A310" t="s">
+        <v>11</v>
+      </c>
+      <c r="B310" t="s">
+        <v>100</v>
+      </c>
+      <c r="C310" t="s">
+        <v>21</v>
+      </c>
+      <c r="D310">
+        <v>10000</v>
+      </c>
+      <c r="E310">
+        <v>10000</v>
+      </c>
+      <c r="F310">
+        <v>20</v>
+      </c>
+      <c r="G310">
+        <v>10000000</v>
+      </c>
+      <c r="H310">
+        <v>0</v>
+      </c>
+      <c r="I310">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="311" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A311" t="s">
+        <v>11</v>
+      </c>
+      <c r="B311" t="s">
+        <v>100</v>
+      </c>
+      <c r="C311" t="s">
+        <v>23</v>
+      </c>
+      <c r="D311">
+        <v>10000</v>
+      </c>
+      <c r="E311">
+        <v>10000</v>
+      </c>
+      <c r="F311">
+        <v>20</v>
+      </c>
+      <c r="G311">
+        <v>10000000</v>
+      </c>
+      <c r="H311">
+        <v>0</v>
+      </c>
+      <c r="I311">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="312" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A312" t="s">
+        <v>11</v>
+      </c>
+      <c r="B312" t="s">
+        <v>100</v>
+      </c>
+      <c r="C312" t="s">
+        <v>25</v>
+      </c>
+      <c r="D312">
+        <v>10000</v>
+      </c>
+      <c r="E312">
+        <v>10000</v>
+      </c>
+      <c r="F312">
+        <v>20</v>
+      </c>
+      <c r="G312">
+        <v>10000000</v>
+      </c>
+      <c r="H312">
+        <v>0</v>
+      </c>
+      <c r="I312">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="313" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A313" t="s">
+        <v>11</v>
+      </c>
+      <c r="B313" t="s">
+        <v>100</v>
+      </c>
+      <c r="C313" t="s">
+        <v>27</v>
+      </c>
+      <c r="D313">
+        <v>10000</v>
+      </c>
+      <c r="E313">
+        <v>10000</v>
+      </c>
+      <c r="F313">
+        <v>20</v>
+      </c>
+      <c r="G313">
+        <v>10000000</v>
+      </c>
+      <c r="H313">
+        <v>0</v>
+      </c>
+      <c r="I313">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="314" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A314" t="s">
+        <v>11</v>
+      </c>
+      <c r="B314" t="s">
+        <v>100</v>
+      </c>
+      <c r="C314" t="s">
+        <v>29</v>
+      </c>
+      <c r="D314">
+        <v>10000</v>
+      </c>
+      <c r="E314">
+        <v>10000</v>
+      </c>
+      <c r="F314">
+        <v>20</v>
+      </c>
+      <c r="G314">
+        <v>10000000</v>
+      </c>
+      <c r="H314">
+        <v>0</v>
+      </c>
+      <c r="I314">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="315" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A315" t="s">
+        <v>11</v>
+      </c>
+      <c r="B315" t="s">
+        <v>100</v>
+      </c>
+      <c r="C315" t="s">
+        <v>31</v>
+      </c>
+      <c r="D315">
+        <v>10000</v>
+      </c>
+      <c r="E315">
+        <v>10000</v>
+      </c>
+      <c r="F315">
+        <v>20</v>
+      </c>
+      <c r="G315">
+        <v>10000000</v>
+      </c>
+      <c r="H315">
+        <v>0</v>
+      </c>
+      <c r="I315">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="316" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A316" t="s">
+        <v>11</v>
+      </c>
+      <c r="B316" t="s">
+        <v>100</v>
+      </c>
+      <c r="C316" t="s">
+        <v>33</v>
+      </c>
+      <c r="D316">
+        <v>10000</v>
+      </c>
+      <c r="E316">
+        <v>10000</v>
+      </c>
+      <c r="F316">
+        <v>20</v>
+      </c>
+      <c r="G316">
+        <v>10000000</v>
+      </c>
+      <c r="H316">
+        <v>0</v>
+      </c>
+      <c r="I316">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="317" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A317" t="s">
+        <v>11</v>
+      </c>
+      <c r="B317" t="s">
+        <v>100</v>
+      </c>
+      <c r="C317" t="s">
+        <v>35</v>
+      </c>
+      <c r="D317">
+        <v>10000</v>
+      </c>
+      <c r="E317">
+        <v>10000</v>
+      </c>
+      <c r="F317">
+        <v>20</v>
+      </c>
+      <c r="G317">
+        <v>10000000</v>
+      </c>
+      <c r="H317">
+        <v>0</v>
+      </c>
+      <c r="I317">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="318" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A318" t="s">
+        <v>12</v>
+      </c>
+      <c r="B318" t="s">
+        <v>100</v>
+      </c>
+      <c r="C318" t="s">
+        <v>15</v>
+      </c>
+      <c r="D318">
+        <v>10000</v>
+      </c>
+      <c r="E318">
+        <v>10000</v>
+      </c>
+      <c r="F318">
+        <v>100</v>
+      </c>
+      <c r="G318">
+        <v>10000000</v>
+      </c>
+      <c r="H318">
+        <v>1000</v>
+      </c>
+      <c r="I318">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="319" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A319" t="s">
+        <v>12</v>
+      </c>
+      <c r="B319" t="s">
+        <v>100</v>
+      </c>
+      <c r="C319" t="s">
+        <v>17</v>
+      </c>
+      <c r="D319">
+        <v>10000</v>
+      </c>
+      <c r="E319">
+        <v>10000</v>
+      </c>
+      <c r="F319">
+        <v>100</v>
+      </c>
+      <c r="G319">
+        <v>10000000</v>
+      </c>
+      <c r="H319">
+        <v>1000</v>
+      </c>
+      <c r="I319">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="320" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A320" t="s">
+        <v>12</v>
+      </c>
+      <c r="B320" t="s">
+        <v>100</v>
+      </c>
+      <c r="C320" t="s">
+        <v>95</v>
+      </c>
+      <c r="D320">
+        <v>10000</v>
+      </c>
+      <c r="E320">
+        <v>10000</v>
+      </c>
+      <c r="F320">
+        <v>100</v>
+      </c>
+      <c r="G320">
+        <v>10000000</v>
+      </c>
+      <c r="H320">
+        <v>1000</v>
+      </c>
+      <c r="I320">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="321" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A321" t="s">
+        <v>12</v>
+      </c>
+      <c r="B321" t="s">
+        <v>100</v>
+      </c>
+      <c r="C321" t="s">
+        <v>19</v>
+      </c>
+      <c r="D321">
+        <v>10000</v>
+      </c>
+      <c r="E321">
+        <v>10000</v>
+      </c>
+      <c r="F321">
+        <v>100</v>
+      </c>
+      <c r="G321">
+        <v>10000000</v>
+      </c>
+      <c r="H321">
+        <v>1000</v>
+      </c>
+      <c r="I321">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="322" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A322" t="s">
+        <v>12</v>
+      </c>
+      <c r="B322" t="s">
+        <v>100</v>
+      </c>
+      <c r="C322" t="s">
+        <v>21</v>
+      </c>
+      <c r="D322">
+        <v>10000</v>
+      </c>
+      <c r="E322">
+        <v>10000</v>
+      </c>
+      <c r="F322">
+        <v>100</v>
+      </c>
+      <c r="G322">
+        <v>10000000</v>
+      </c>
+      <c r="H322">
+        <v>1000</v>
+      </c>
+      <c r="I322">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="323" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A323" t="s">
+        <v>12</v>
+      </c>
+      <c r="B323" t="s">
+        <v>100</v>
+      </c>
+      <c r="C323" t="s">
+        <v>23</v>
+      </c>
+      <c r="D323">
+        <v>10000</v>
+      </c>
+      <c r="E323">
+        <v>10000</v>
+      </c>
+      <c r="F323">
+        <v>100</v>
+      </c>
+      <c r="G323">
+        <v>10000000</v>
+      </c>
+      <c r="H323">
+        <v>1000</v>
+      </c>
+      <c r="I323">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="324" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A324" t="s">
+        <v>12</v>
+      </c>
+      <c r="B324" t="s">
+        <v>100</v>
+      </c>
+      <c r="C324" t="s">
+        <v>25</v>
+      </c>
+      <c r="D324">
+        <v>10000</v>
+      </c>
+      <c r="E324">
+        <v>10000</v>
+      </c>
+      <c r="F324">
+        <v>100</v>
+      </c>
+      <c r="G324">
+        <v>10000000</v>
+      </c>
+      <c r="H324">
+        <v>1000</v>
+      </c>
+      <c r="I324">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="325" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A325" t="s">
+        <v>12</v>
+      </c>
+      <c r="B325" t="s">
+        <v>100</v>
+      </c>
+      <c r="C325" t="s">
+        <v>27</v>
+      </c>
+      <c r="D325">
+        <v>10000</v>
+      </c>
+      <c r="E325">
+        <v>10000</v>
+      </c>
+      <c r="F325">
+        <v>100</v>
+      </c>
+      <c r="G325">
+        <v>10000000</v>
+      </c>
+      <c r="H325">
+        <v>1000</v>
+      </c>
+      <c r="I325">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="326" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A326" t="s">
+        <v>12</v>
+      </c>
+      <c r="B326" t="s">
+        <v>100</v>
+      </c>
+      <c r="C326" t="s">
+        <v>29</v>
+      </c>
+      <c r="D326">
+        <v>10000</v>
+      </c>
+      <c r="E326">
+        <v>10000</v>
+      </c>
+      <c r="F326">
+        <v>100</v>
+      </c>
+      <c r="G326">
+        <v>10000000</v>
+      </c>
+      <c r="H326">
+        <v>1000</v>
+      </c>
+      <c r="I326">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="327" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A327" t="s">
+        <v>12</v>
+      </c>
+      <c r="B327" t="s">
+        <v>100</v>
+      </c>
+      <c r="C327" t="s">
+        <v>31</v>
+      </c>
+      <c r="D327">
+        <v>10000</v>
+      </c>
+      <c r="E327">
+        <v>10000</v>
+      </c>
+      <c r="F327">
+        <v>100</v>
+      </c>
+      <c r="G327">
+        <v>10000000</v>
+      </c>
+      <c r="H327">
+        <v>1000</v>
+      </c>
+      <c r="I327">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="328" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A328" t="s">
+        <v>12</v>
+      </c>
+      <c r="B328" t="s">
+        <v>100</v>
+      </c>
+      <c r="C328" t="s">
+        <v>33</v>
+      </c>
+      <c r="D328">
+        <v>10000</v>
+      </c>
+      <c r="E328">
+        <v>10000</v>
+      </c>
+      <c r="F328">
+        <v>100</v>
+      </c>
+      <c r="G328">
+        <v>10000000</v>
+      </c>
+      <c r="H328">
+        <v>1000</v>
+      </c>
+      <c r="I328">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="329" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A329" t="s">
+        <v>12</v>
+      </c>
+      <c r="B329" t="s">
+        <v>100</v>
+      </c>
+      <c r="C329" t="s">
+        <v>35</v>
+      </c>
+      <c r="D329">
+        <v>10000</v>
+      </c>
+      <c r="E329">
+        <v>10000</v>
+      </c>
+      <c r="F329">
+        <v>100</v>
+      </c>
+      <c r="G329">
+        <v>10000000</v>
+      </c>
+      <c r="H329">
+        <v>1000</v>
+      </c>
+      <c r="I329">
         <v>1</v>
       </c>
     </row>
@@ -10629,7 +12313,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C68B577B-1347-43AB-A697-F4519763B965}">
-  <dimension ref="A1:C170"/>
+  <dimension ref="A1:C242"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -10651,7 +12335,7 @@
         <v>15</v>
       </c>
       <c r="C2">
-        <v>111.378</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -10662,7 +12346,7 @@
         <v>17</v>
       </c>
       <c r="C3">
-        <v>322.40999999999997</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -10673,7 +12357,7 @@
         <v>95</v>
       </c>
       <c r="C4">
-        <v>73.274999999999991</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -10684,7 +12368,7 @@
         <v>19</v>
       </c>
       <c r="C5">
-        <v>155.83149999999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
@@ -10695,7 +12379,7 @@
         <v>21</v>
       </c>
       <c r="C6">
-        <v>25.402000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
@@ -10706,7 +12390,7 @@
         <v>23</v>
       </c>
       <c r="C7">
-        <v>39.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
@@ -10717,7 +12401,7 @@
         <v>25</v>
       </c>
       <c r="C8">
-        <v>122.125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
@@ -10728,7 +12412,7 @@
         <v>27</v>
       </c>
       <c r="C9">
-        <v>60.573999999999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
@@ -10739,7 +12423,7 @@
         <v>29</v>
       </c>
       <c r="C10">
-        <v>74.251999999999995</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
@@ -10750,7 +12434,7 @@
         <v>31</v>
       </c>
       <c r="C11">
-        <v>655.56699999999989</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
@@ -10761,7 +12445,7 @@
         <v>33</v>
       </c>
       <c r="C12">
-        <v>425.97199999999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
@@ -10772,7 +12456,7 @@
         <v>35</v>
       </c>
       <c r="C13">
-        <v>510.97099999999995</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
@@ -12499,6 +14183,699 @@
         <v>68</v>
       </c>
       <c r="C170">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A171" t="s">
+        <v>11</v>
+      </c>
+      <c r="B171" t="s">
+        <v>99</v>
+      </c>
+      <c r="C171">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A172" t="s">
+        <v>11</v>
+      </c>
+      <c r="B172" t="s">
+        <v>98</v>
+      </c>
+      <c r="C172">
+        <v>-1000</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A173" t="s">
+        <v>11</v>
+      </c>
+      <c r="B173" t="s">
+        <v>100</v>
+      </c>
+      <c r="C173">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A174" t="s">
+        <v>12</v>
+      </c>
+      <c r="B174" t="s">
+        <v>99</v>
+      </c>
+      <c r="C174">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A175" t="s">
+        <v>12</v>
+      </c>
+      <c r="B175" t="s">
+        <v>98</v>
+      </c>
+      <c r="C175">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A176" t="s">
+        <v>12</v>
+      </c>
+      <c r="B176" t="s">
+        <v>100</v>
+      </c>
+      <c r="C176">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A177" t="s">
+        <v>11</v>
+      </c>
+      <c r="B177" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A178" t="s">
+        <v>11</v>
+      </c>
+      <c r="B178" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A179" t="s">
+        <v>11</v>
+      </c>
+      <c r="B179" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A180" t="s">
+        <v>11</v>
+      </c>
+      <c r="B180" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A181" t="s">
+        <v>11</v>
+      </c>
+      <c r="B181" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A182" t="s">
+        <v>11</v>
+      </c>
+      <c r="B182" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A183" t="s">
+        <v>11</v>
+      </c>
+      <c r="B183" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A184" t="s">
+        <v>11</v>
+      </c>
+      <c r="B184" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A185" t="s">
+        <v>11</v>
+      </c>
+      <c r="B185" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A186" t="s">
+        <v>11</v>
+      </c>
+      <c r="B186" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A187" t="s">
+        <v>11</v>
+      </c>
+      <c r="B187" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A188" t="s">
+        <v>11</v>
+      </c>
+      <c r="B188" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A189" t="s">
+        <v>11</v>
+      </c>
+      <c r="B189" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A190" t="s">
+        <v>11</v>
+      </c>
+      <c r="B190" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A191" t="s">
+        <v>11</v>
+      </c>
+      <c r="B191" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A192" t="s">
+        <v>11</v>
+      </c>
+      <c r="B192" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A193" t="s">
+        <v>11</v>
+      </c>
+      <c r="B193" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A194" t="s">
+        <v>11</v>
+      </c>
+      <c r="B194" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A195" t="s">
+        <v>11</v>
+      </c>
+      <c r="B195" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A196" t="s">
+        <v>11</v>
+      </c>
+      <c r="B196" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A197" t="s">
+        <v>11</v>
+      </c>
+      <c r="B197" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A198" t="s">
+        <v>11</v>
+      </c>
+      <c r="B198" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A199" t="s">
+        <v>11</v>
+      </c>
+      <c r="B199" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A200" t="s">
+        <v>11</v>
+      </c>
+      <c r="B200" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A201" t="s">
+        <v>11</v>
+      </c>
+      <c r="B201" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A202" t="s">
+        <v>11</v>
+      </c>
+      <c r="B202" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A203" t="s">
+        <v>11</v>
+      </c>
+      <c r="B203" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A204" t="s">
+        <v>11</v>
+      </c>
+      <c r="B204" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A205" t="s">
+        <v>11</v>
+      </c>
+      <c r="B205" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A206" t="s">
+        <v>11</v>
+      </c>
+      <c r="B206" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A207" t="s">
+        <v>11</v>
+      </c>
+      <c r="B207" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A208" t="s">
+        <v>11</v>
+      </c>
+      <c r="B208" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="209" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A209" t="s">
+        <v>11</v>
+      </c>
+      <c r="B209" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A210" t="s">
+        <v>12</v>
+      </c>
+      <c r="B210" t="s">
+        <v>102</v>
+      </c>
+      <c r="C210">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A211" t="s">
+        <v>12</v>
+      </c>
+      <c r="B211" t="s">
+        <v>101</v>
+      </c>
+      <c r="C211">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A212" t="s">
+        <v>12</v>
+      </c>
+      <c r="B212" t="s">
+        <v>103</v>
+      </c>
+      <c r="C212">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A213" t="s">
+        <v>12</v>
+      </c>
+      <c r="B213" t="s">
+        <v>104</v>
+      </c>
+      <c r="C213">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A214" t="s">
+        <v>12</v>
+      </c>
+      <c r="B214" t="s">
+        <v>105</v>
+      </c>
+      <c r="C214">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A215" t="s">
+        <v>12</v>
+      </c>
+      <c r="B215" t="s">
+        <v>106</v>
+      </c>
+      <c r="C215">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A216" t="s">
+        <v>12</v>
+      </c>
+      <c r="B216" t="s">
+        <v>107</v>
+      </c>
+      <c r="C216">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A217" t="s">
+        <v>12</v>
+      </c>
+      <c r="B217" t="s">
+        <v>108</v>
+      </c>
+      <c r="C217">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A218" t="s">
+        <v>12</v>
+      </c>
+      <c r="B218" t="s">
+        <v>109</v>
+      </c>
+      <c r="C218">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A219" t="s">
+        <v>12</v>
+      </c>
+      <c r="B219" t="s">
+        <v>110</v>
+      </c>
+      <c r="C219">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A220" t="s">
+        <v>12</v>
+      </c>
+      <c r="B220" t="s">
+        <v>111</v>
+      </c>
+      <c r="C220">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A221" t="s">
+        <v>12</v>
+      </c>
+      <c r="B221" t="s">
+        <v>112</v>
+      </c>
+      <c r="C221">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A222" t="s">
+        <v>12</v>
+      </c>
+      <c r="B222" t="s">
+        <v>113</v>
+      </c>
+      <c r="C222">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A223" t="s">
+        <v>12</v>
+      </c>
+      <c r="B223" t="s">
+        <v>114</v>
+      </c>
+      <c r="C223">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A224" t="s">
+        <v>12</v>
+      </c>
+      <c r="B224" t="s">
+        <v>115</v>
+      </c>
+      <c r="C224">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A225" t="s">
+        <v>12</v>
+      </c>
+      <c r="B225" t="s">
+        <v>116</v>
+      </c>
+      <c r="C225">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A226" t="s">
+        <v>12</v>
+      </c>
+      <c r="B226" t="s">
+        <v>117</v>
+      </c>
+      <c r="C226">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A227" t="s">
+        <v>12</v>
+      </c>
+      <c r="B227" t="s">
+        <v>118</v>
+      </c>
+      <c r="C227">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A228" t="s">
+        <v>12</v>
+      </c>
+      <c r="B228" t="s">
+        <v>119</v>
+      </c>
+      <c r="C228">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="229" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A229" t="s">
+        <v>12</v>
+      </c>
+      <c r="B229" t="s">
+        <v>120</v>
+      </c>
+      <c r="C229">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="230" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A230" t="s">
+        <v>12</v>
+      </c>
+      <c r="B230" t="s">
+        <v>121</v>
+      </c>
+      <c r="C230">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="231" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A231" t="s">
+        <v>12</v>
+      </c>
+      <c r="B231" t="s">
+        <v>122</v>
+      </c>
+      <c r="C231">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="232" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A232" t="s">
+        <v>12</v>
+      </c>
+      <c r="B232" t="s">
+        <v>123</v>
+      </c>
+      <c r="C232">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A233" t="s">
+        <v>12</v>
+      </c>
+      <c r="B233" t="s">
+        <v>124</v>
+      </c>
+      <c r="C233">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="234" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A234" t="s">
+        <v>12</v>
+      </c>
+      <c r="B234" t="s">
+        <v>125</v>
+      </c>
+      <c r="C234">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="235" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A235" t="s">
+        <v>12</v>
+      </c>
+      <c r="B235" t="s">
+        <v>126</v>
+      </c>
+      <c r="C235">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="236" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A236" t="s">
+        <v>12</v>
+      </c>
+      <c r="B236" t="s">
+        <v>127</v>
+      </c>
+      <c r="C236">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="237" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A237" t="s">
+        <v>12</v>
+      </c>
+      <c r="B237" t="s">
+        <v>128</v>
+      </c>
+      <c r="C237">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="238" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A238" t="s">
+        <v>12</v>
+      </c>
+      <c r="B238" t="s">
+        <v>129</v>
+      </c>
+      <c r="C238">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="239" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A239" t="s">
+        <v>12</v>
+      </c>
+      <c r="B239" t="s">
+        <v>130</v>
+      </c>
+      <c r="C239">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="240" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A240" t="s">
+        <v>12</v>
+      </c>
+      <c r="B240" t="s">
+        <v>131</v>
+      </c>
+      <c r="C240">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="241" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A241" t="s">
+        <v>12</v>
+      </c>
+      <c r="B241" t="s">
+        <v>132</v>
+      </c>
+      <c r="C241">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="242" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A242" t="s">
+        <v>12</v>
+      </c>
+      <c r="B242" t="s">
+        <v>133</v>
+      </c>
+      <c r="C242">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
model testing and bug identification
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/data_case_russia_BASE.xlsx
+++ b/01_data/01_input_data/02_processed/data_case_russia_BASE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAC617E2-61F9-4316-B75B-582595AA4FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B767F2F6-3EEF-41EB-B557-CD1B72D02024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
@@ -15292,7 +15292,7 @@
         <v>10000</v>
       </c>
       <c r="F373">
-        <v>2020.2037108265431</v>
+        <v>22.203710826543102</v>
       </c>
       <c r="G373">
         <v>10000000</v>
@@ -15321,7 +15321,7 @@
         <v>10000</v>
       </c>
       <c r="F374">
-        <v>2014.7448142896919</v>
+        <v>16.744814289691931</v>
       </c>
       <c r="G374">
         <v>10000000</v>
@@ -15350,7 +15350,7 @@
         <v>10000</v>
       </c>
       <c r="F375">
-        <v>2011.80615123654</v>
+        <v>13.806151236540018</v>
       </c>
       <c r="G375">
         <v>10000000</v>
@@ -15379,7 +15379,7 @@
         <v>10000</v>
       </c>
       <c r="F376">
-        <v>2014.329603409235</v>
+        <v>16.329603409235006</v>
       </c>
       <c r="G376">
         <v>10000000</v>
@@ -15408,7 +15408,7 @@
         <v>10000</v>
       </c>
       <c r="F377">
-        <v>2013.9272672847619</v>
+        <v>15.927267284761911</v>
       </c>
       <c r="G377">
         <v>10000000</v>
@@ -15437,7 +15437,7 @@
         <v>10000</v>
       </c>
       <c r="F378">
-        <v>2023.209966348606</v>
+        <v>25.209966348606031</v>
       </c>
       <c r="G378">
         <v>10000000</v>
@@ -15466,7 +15466,7 @@
         <v>10000</v>
       </c>
       <c r="F379">
-        <v>2020.4258003672519</v>
+        <v>22.425800367251895</v>
       </c>
       <c r="G379">
         <v>10000000</v>
@@ -15495,7 +15495,7 @@
         <v>10000</v>
       </c>
       <c r="F380">
-        <v>2022.595196750412</v>
+        <v>24.595196750412015</v>
       </c>
       <c r="G380">
         <v>10000000</v>
@@ -15524,7 +15524,7 @@
         <v>10000</v>
       </c>
       <c r="F381">
-        <v>2016.9496162518039</v>
+        <v>18.949616251803945</v>
       </c>
       <c r="G381">
         <v>10000000</v>
@@ -15553,7 +15553,7 @@
         <v>10000</v>
       </c>
       <c r="F382">
-        <v>2014.9894346533711</v>
+        <v>16.989434653371063</v>
       </c>
       <c r="G382">
         <v>10000000</v>
@@ -15582,7 +15582,7 @@
         <v>10000</v>
       </c>
       <c r="F383">
-        <v>2011.8029325475441</v>
+        <v>13.80293254754406</v>
       </c>
       <c r="G383">
         <v>10000000</v>
@@ -15611,7 +15611,7 @@
         <v>10000</v>
       </c>
       <c r="F384">
-        <v>2019.6050346733271</v>
+        <v>21.605034673327054</v>
       </c>
       <c r="G384">
         <v>10000000</v>

</xml_diff>